<commit_message>
chore: update piezo stats
</commit_message>
<xml_diff>
--- a/Data/Piezo stats.xlsx
+++ b/Data/Piezo stats.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Pesquisa\Piezo stack actuator\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3413FE79-A047-4B6E-903E-4E20FF902574}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2C25BB6-5957-41FD-A1BE-2FAD376E097A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{28825E0A-C981-4FF2-8652-165F0953E153}"/>
   </bookViews>
@@ -3499,6 +3499,7 @@
       <formula1>"caliper,micrometer,multimeter"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.78740157480314965" bottom="0.78740157480314965" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" scale="47" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>